<commit_message>
Database: contact points, recreate scripts, tenant seed; update docs
- Schema/migration: fnd_contact_points, recreate_all*, seed_fnd_tenants
- Docs: Obsidian workspace, BPS Tables workbook

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/BPS Tables.xlsx
+++ b/docs/BPS Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\orderNexa\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5844749-1FA1-448F-85C9-1214A2565328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B4024C-DAA3-4D04-8E4B-15FCCCB5DA26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-1850" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{04488C40-F022-43DD-81A9-CABA93E3C950}"/>
+    <workbookView xWindow="19090" yWindow="-1850" windowWidth="25820" windowHeight="15500" xr2:uid="{04488C40-F022-43DD-81A9-CABA93E3C950}"/>
   </bookViews>
   <sheets>
     <sheet name="tenant &amp; User" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="FND" sheetId="13" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -932,15 +933,6 @@
     <t>is_Active</t>
   </si>
   <si>
-    <t>entity_id</t>
-  </si>
-  <si>
-    <t>FND_PEOPLE</t>
-  </si>
-  <si>
-    <t>person_id</t>
-  </si>
-  <si>
     <t>is_primary</t>
   </si>
   <si>
@@ -993,13 +985,22 @@
   </si>
   <si>
     <t>om_order_production</t>
+  </si>
+  <si>
+    <t>FND_CONTACTS</t>
+  </si>
+  <si>
+    <t>contact_id</t>
+  </si>
+  <si>
+    <t>contact_point_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1129,6 +1130,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1380,7 +1389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1532,6 +1541,30 @@
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1556,6 +1589,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1574,35 +1613,8 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2051,7 +2063,7 @@
     <col min="12" max="12" width="17.7109375" style="47" customWidth="1"/>
     <col min="13" max="13" width="12.42578125" style="47" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="23" style="47" customWidth="1"/>
-    <col min="15" max="15" width="18.5703125" style="47" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" style="47" bestFit="1" customWidth="1"/>
     <col min="16" max="16384" width="9.140625" style="47"/>
   </cols>
   <sheetData>
@@ -2066,10 +2078,10 @@
         <v>270</v>
       </c>
       <c r="D1" s="49" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="E1" s="49" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="F1" s="46" t="s">
         <v>273</v>
@@ -2090,11 +2102,11 @@
       <c r="L1" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="N1" s="48" t="s">
-        <v>297</v>
+      <c r="N1" s="75" t="s">
+        <v>314</v>
       </c>
       <c r="O1" s="48" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -2108,10 +2120,10 @@
         <v>271</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E2" s="47" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F2" s="47" t="s">
         <v>271</v>
@@ -2132,10 +2144,10 @@
         <v>11</v>
       </c>
       <c r="N2" s="47" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="O2" s="47" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2143,7 +2155,7 @@
         <v>190</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D3" s="47" t="s">
         <v>104</v>
@@ -2170,10 +2182,10 @@
         <v>122</v>
       </c>
       <c r="N3" s="47" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="O3" s="47" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -2190,15 +2202,15 @@
         <v>283</v>
       </c>
       <c r="N4" s="47" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="O4" s="47" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C5" s="47" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>134</v>
@@ -2207,10 +2219,10 @@
         <v>104</v>
       </c>
       <c r="N5" s="47" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="O5" s="47" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -2218,18 +2230,18 @@
         <v>295</v>
       </c>
       <c r="D6" s="47" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E6" s="47" t="s">
         <v>134</v>
       </c>
       <c r="N6" s="47" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="N7" s="47" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2239,7 +2251,7 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="N9" s="47" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2355,30 +2367,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="61" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="D1" s="53" t="s">
+      <c r="B1" s="62"/>
+      <c r="D1" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="G1" s="57" t="s">
+      <c r="E1" s="62"/>
+      <c r="G1" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="58"/>
-      <c r="J1" s="57" t="s">
+      <c r="H1" s="66"/>
+      <c r="J1" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="58"/>
-      <c r="M1" s="72" t="s">
-        <v>316</v>
-      </c>
-      <c r="N1" s="73"/>
-      <c r="P1" s="55" t="s">
+      <c r="K1" s="66"/>
+      <c r="M1" s="67" t="s">
+        <v>313</v>
+      </c>
+      <c r="N1" s="68"/>
+      <c r="P1" s="63" t="s">
         <v>250</v>
       </c>
-      <c r="Q1" s="56"/>
+      <c r="Q1" s="64"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
@@ -2399,14 +2411,14 @@
       <c r="H2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="52" t="s">
         <v>72</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="M2" s="68"/>
-      <c r="N2" s="69"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="55"/>
       <c r="P2" s="37" t="s">
         <v>253</v>
       </c>
@@ -2439,8 +2451,8 @@
       <c r="K3" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="M3" s="68"/>
-      <c r="N3" s="69"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="55"/>
       <c r="P3" s="36" t="s">
         <v>9</v>
       </c>
@@ -2473,9 +2485,9 @@
       <c r="K4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="M4" s="68"/>
-      <c r="N4" s="69"/>
-      <c r="P4" s="65" t="s">
+      <c r="M4" s="54"/>
+      <c r="N4" s="55"/>
+      <c r="P4" s="51" t="s">
         <v>72</v>
       </c>
       <c r="Q4" s="5" t="s">
@@ -2507,8 +2519,8 @@
       <c r="K5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="M5" s="68"/>
-      <c r="N5" s="69"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="55"/>
       <c r="P5" s="24" t="s">
         <v>251</v>
       </c>
@@ -2541,8 +2553,8 @@
       <c r="K6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="68"/>
-      <c r="N6" s="69"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="55"/>
       <c r="P6" s="4" t="s">
         <v>2</v>
       </c>
@@ -2575,8 +2587,8 @@
       <c r="K7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="68"/>
-      <c r="N7" s="69"/>
+      <c r="M7" s="54"/>
+      <c r="N7" s="55"/>
       <c r="P7" s="36" t="s">
         <v>254</v>
       </c>
@@ -2609,8 +2621,8 @@
       <c r="K8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="68"/>
-      <c r="N8" s="69"/>
+      <c r="M8" s="54"/>
+      <c r="N8" s="55"/>
       <c r="P8" s="38" t="s">
         <v>252</v>
       </c>
@@ -2631,8 +2643,8 @@
       <c r="E9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="67" t="s">
-        <v>315</v>
+      <c r="G9" s="53" t="s">
+        <v>312</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>23</v>
@@ -2643,8 +2655,8 @@
       <c r="K9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="68"/>
-      <c r="N9" s="69"/>
+      <c r="M9" s="54"/>
+      <c r="N9" s="55"/>
       <c r="P9" s="4" t="s">
         <v>255</v>
       </c>
@@ -2677,9 +2689,9 @@
       <c r="K10" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="M10" s="70"/>
-      <c r="N10" s="71"/>
-      <c r="P10" s="74" t="s">
+      <c r="M10" s="56"/>
+      <c r="N10" s="57"/>
+      <c r="P10" s="58" t="s">
         <v>98</v>
       </c>
       <c r="Q10" s="27" t="s">
@@ -2705,8 +2717,8 @@
       <c r="H11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="P11" s="74" t="s">
-        <v>315</v>
+      <c r="P11" s="58" t="s">
+        <v>312</v>
       </c>
       <c r="Q11" s="27" t="s">
         <v>23</v>
@@ -2786,33 +2798,33 @@
       <c r="B16" s="1"/>
     </row>
     <row r="17" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="53" t="s">
+      <c r="A17" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="54"/>
-      <c r="D17" s="53" t="s">
+      <c r="B17" s="62"/>
+      <c r="D17" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="54"/>
-      <c r="G17" s="51" t="s">
+      <c r="E17" s="62"/>
+      <c r="G17" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="H17" s="52"/>
-      <c r="J17" s="51" t="s">
+      <c r="H17" s="60"/>
+      <c r="J17" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="K17" s="52"/>
-      <c r="M17" s="51" t="s">
+      <c r="K17" s="60"/>
+      <c r="M17" s="59" t="s">
         <v>267</v>
       </c>
-      <c r="N17" s="52"/>
+      <c r="N17" s="60"/>
       <c r="O17" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="P17" s="51" t="s">
+      <c r="P17" s="59" t="s">
         <v>264</v>
       </c>
-      <c r="Q17" s="52"/>
+      <c r="Q17" s="60"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
@@ -3165,10 +3177,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="60"/>
+      <c r="B1" s="70"/>
     </row>
     <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -3255,10 +3267,10 @@
       <c r="B13" s="34"/>
     </row>
     <row r="14" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="60"/>
+      <c r="B14" s="70"/>
     </row>
     <row r="15" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
@@ -3355,10 +3367,10 @@
       <c r="B27" s="34"/>
     </row>
     <row r="28" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="B28" s="60"/>
+      <c r="B28" s="70"/>
     </row>
     <row r="29" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
@@ -3425,10 +3437,10 @@
       <c r="B37" s="34"/>
     </row>
     <row r="38" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="B38" s="60"/>
+      <c r="B38" s="70"/>
     </row>
     <row r="39" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
@@ -3503,10 +3515,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="62"/>
+      <c r="B1" s="72"/>
     </row>
     <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -3611,10 +3623,10 @@
       <c r="B15" s="34"/>
     </row>
     <row r="16" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="61" t="s">
+      <c r="A16" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="62"/>
+      <c r="B16" s="72"/>
     </row>
     <row r="17" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
@@ -3695,10 +3707,10 @@
       <c r="B27" s="34"/>
     </row>
     <row r="28" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="61" t="s">
+      <c r="A28" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="B28" s="62"/>
+      <c r="B28" s="72"/>
     </row>
     <row r="29" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
@@ -3800,10 +3812,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="73" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="64"/>
+      <c r="B1" s="74"/>
     </row>
     <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -3842,10 +3854,10 @@
       <c r="B7" s="34"/>
     </row>
     <row r="8" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="73" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="64"/>
+      <c r="B8" s="74"/>
     </row>
     <row r="9" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="33" t="s">
@@ -3976,10 +3988,10 @@
       <c r="B25" s="34"/>
     </row>
     <row r="26" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="73" t="s">
         <v>195</v>
       </c>
-      <c r="B26" s="64"/>
+      <c r="B26" s="74"/>
     </row>
     <row r="27" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
@@ -4048,10 +4060,10 @@
       <c r="B37" s="34"/>
     </row>
     <row r="38" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="63" t="s">
+      <c r="A38" s="73" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="64"/>
+      <c r="B38" s="74"/>
     </row>
     <row r="39" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
@@ -4196,10 +4208,10 @@
       <c r="B57" s="34"/>
     </row>
     <row r="58" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="63" t="s">
+      <c r="A58" s="73" t="s">
         <v>207</v>
       </c>
-      <c r="B58" s="64"/>
+      <c r="B58" s="74"/>
     </row>
     <row r="59" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="33" t="s">
@@ -4244,10 +4256,10 @@
       <c r="B65" s="34"/>
     </row>
     <row r="66" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="63" t="s">
+      <c r="A66" s="73" t="s">
         <v>169</v>
       </c>
-      <c r="B66" s="64"/>
+      <c r="B66" s="74"/>
     </row>
     <row r="67" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
@@ -4296,10 +4308,10 @@
       <c r="B73" s="34"/>
     </row>
     <row r="74" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="63" t="s">
+      <c r="A74" s="73" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="64"/>
+      <c r="B74" s="74"/>
     </row>
     <row r="75" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
@@ -4362,10 +4374,10 @@
       <c r="B83" s="34"/>
     </row>
     <row r="84" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="63" t="s">
+      <c r="A84" s="73" t="s">
         <v>171</v>
       </c>
-      <c r="B84" s="64"/>
+      <c r="B84" s="74"/>
     </row>
     <row r="85" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
@@ -4426,10 +4438,10 @@
       <c r="B93" s="34"/>
     </row>
     <row r="94" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="63" t="s">
+      <c r="A94" s="73" t="s">
         <v>175</v>
       </c>
-      <c r="B94" s="64"/>
+      <c r="B94" s="74"/>
     </row>
     <row r="95" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="33" t="s">

</xml_diff>

<commit_message>
Database and order management updates across function naming, policies, and API integration.
Align SQL function and migration assets with the new naming convention and refresh tenant/order entry flows in the web app to match the updated backend contracts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/BPS Tables.xlsx
+++ b/docs/BPS Tables.xlsx
@@ -8,17 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\orderNexa\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B4024C-DAA3-4D04-8E4B-15FCCCB5DA26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4028A179-4A93-442D-994C-9D225303FC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-1850" windowWidth="25820" windowHeight="15500" xr2:uid="{04488C40-F022-43DD-81A9-CABA93E3C950}"/>
+    <workbookView xWindow="19090" yWindow="-1850" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{04488C40-F022-43DD-81A9-CABA93E3C950}"/>
   </bookViews>
   <sheets>
     <sheet name="tenant &amp; User" sheetId="1" r:id="rId1"/>
     <sheet name="FND_ITEMS" sheetId="17" r:id="rId2"/>
     <sheet name="Order &amp; AR" sheetId="2" r:id="rId3"/>
     <sheet name="AR" sheetId="12" r:id="rId4"/>
-    <sheet name="OM" sheetId="14" r:id="rId5"/>
-    <sheet name="FND" sheetId="13" r:id="rId6"/>
+    <sheet name="FND" sheetId="13" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="290">
   <si>
     <t>ar_transactions</t>
   </si>
@@ -83,9 +82,6 @@
     <t>order_date</t>
   </si>
   <si>
-    <t>delivery_date</t>
-  </si>
-  <si>
     <t>ordr</t>
   </si>
   <si>
@@ -320,30 +316,15 @@
     <t>extended_amount</t>
   </si>
   <si>
-    <t>om_order_fullfillments</t>
-  </si>
-  <si>
     <t>order_fulfillment_id</t>
   </si>
   <si>
-    <t>fulfillment_type</t>
-  </si>
-  <si>
-    <t>occurred_at</t>
-  </si>
-  <si>
     <t>timestamp</t>
   </si>
   <si>
-    <t>delivery_window</t>
-  </si>
-  <si>
     <t>production_date</t>
   </si>
   <si>
-    <t>production_window</t>
-  </si>
-  <si>
     <t>bigInt</t>
   </si>
   <si>
@@ -359,36 +340,9 @@
     <t>tenant_id</t>
   </si>
   <si>
-    <t>ordr.ordr_no</t>
-  </si>
-  <si>
-    <t>ordr.ordr_prdctn_cd</t>
-  </si>
-  <si>
-    <t>ordr.ordr_amt</t>
-  </si>
-  <si>
-    <t>ordr.ordr_discount_amt</t>
-  </si>
-  <si>
-    <t>ordr.ordr_qty_sold</t>
-  </si>
-  <si>
     <t>Source (table.column)</t>
   </si>
   <si>
-    <t>ordr_detail.item_desc</t>
-  </si>
-  <si>
-    <t>ordr_detail.od_qty_sold</t>
-  </si>
-  <si>
-    <t>ordr_detail.od_item_cost</t>
-  </si>
-  <si>
-    <t>ordr_detail.od_item_discount</t>
-  </si>
-  <si>
     <t>pmt_detail.pd_pmt_no</t>
   </si>
   <si>
@@ -578,24 +532,6 @@
     <t>citem.citem_qty</t>
   </si>
   <si>
-    <t>ordr.ordr_prdctn_dt</t>
-  </si>
-  <si>
-    <t>ordr.ordr_prdctn_dt, ordr.ordr_dt</t>
-  </si>
-  <si>
-    <t>ordr.cus_name, ordr.cus_key, ordr.route_id, ordr.route_stop_no, customer.cus_invc_rqrd, customer.cus_dlvr_instr, customer.cus_parent_id, customer.cus_id, customer.s_contact, customer.s_addr1, customer.s_addr2, customer.s_city, customer.s_state, customer.s_zip, customer.b_contact, customer.b_addr1, customer.b_addr2, customer.b_city, customer.b_state, customer.b_zip</t>
-  </si>
-  <si>
-    <t>fulfilled_quantity</t>
-  </si>
-  <si>
-    <t>ordr_detail.ordr_no, ordr_detail.od_qty_sold</t>
-  </si>
-  <si>
-    <t>ordr.cus_id, fnd_customers.legacy_id, fnd_customers.customer_id</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -605,9 +541,6 @@
     <t>source_type</t>
   </si>
   <si>
-    <t>ordr_detail.item_id, fnd_items.legacy_id, fnd_items.item_id</t>
-  </si>
-  <si>
     <t>om_order_fullfillments.order_fulfillment_id</t>
   </si>
   <si>
@@ -731,18 +664,6 @@
     <t>citem.item_id, fnd_items.legacy_id, fnd_items.item_id</t>
   </si>
   <si>
-    <t>ordr_detail.ordr_no, om_orders.order_number, om_orders.order_id</t>
-  </si>
-  <si>
-    <t>ordr_detail.item_id, fnd_items.legacy_id, fnd_items.item_id, om_order_lines.item_id, om_order_lines.order_line_id</t>
-  </si>
-  <si>
-    <t>om_orders.delivery_date, om_orders.order_date</t>
-  </si>
-  <si>
-    <t>om_orders.delivery_window</t>
-  </si>
-  <si>
     <t>om_orders.customer_id</t>
   </si>
   <si>
@@ -789,10 +710,6 @@
   </si>
   <si>
     <t>pmt_detail.pd_ar_trn_id, ar_transactions.legacy_ar_id, ar_transactions.ar_transaction_id</t>
-  </si>
-  <si>
-    <t>unit_discount
-discount_amount</t>
   </si>
   <si>
     <t>om_order_shipments</t>
@@ -1000,7 +917,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1094,12 +1011,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color theme="6"/>
@@ -1143,7 +1054,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1177,12 +1088,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDFEEFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDFF5DF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1389,7 +1294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1493,9 +1398,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1520,13 +1422,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1535,36 +1437,36 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1601,19 +1503,13 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2051,280 +1947,255 @@
   <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" style="47" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" style="47" customWidth="1"/>
-    <col min="3" max="4" width="17.42578125" style="47" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.42578125" style="47" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" style="47" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" style="47" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23" style="47" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="47" customWidth="1"/>
-    <col min="12" max="12" width="17.7109375" style="47" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" style="47" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23" style="47" customWidth="1"/>
-    <col min="15" max="15" width="22.5703125" style="47" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="47"/>
+    <col min="1" max="1" width="19.28515625" style="46" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" style="46" customWidth="1"/>
+    <col min="3" max="4" width="17.42578125" style="46" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" style="46" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.42578125" style="46" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" style="46" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23" style="46" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="46" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="46" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" style="46" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23" style="46" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" style="46" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="46"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
-        <v>189</v>
-      </c>
-      <c r="B1" s="49" t="s">
-        <v>189</v>
-      </c>
-      <c r="C1" s="49" t="s">
+      <c r="A1" s="48" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="48" t="s">
+        <v>243</v>
+      </c>
+      <c r="D1" s="48" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1" s="48" t="s">
+        <v>279</v>
+      </c>
+      <c r="F1" s="45" t="s">
+        <v>246</v>
+      </c>
+      <c r="G1" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="H1" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="I1" s="45" t="s">
+        <v>257</v>
+      </c>
+      <c r="J1" s="45" t="s">
+        <v>260</v>
+      </c>
+      <c r="K1" s="45"/>
+      <c r="L1" s="49" t="s">
+        <v>102</v>
+      </c>
+      <c r="N1" s="72" t="s">
+        <v>287</v>
+      </c>
+      <c r="O1" s="47" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="G2" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="H2" s="46" t="s">
+        <v>254</v>
+      </c>
+      <c r="I2" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="J2" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="L2" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="46" t="s">
+        <v>288</v>
+      </c>
+      <c r="O2" s="46" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="G3" s="46" t="s">
+        <v>250</v>
+      </c>
+      <c r="H3" s="46" t="s">
+        <v>255</v>
+      </c>
+      <c r="I3" s="46" t="s">
+        <v>259</v>
+      </c>
+      <c r="J3" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="N3" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="O3" s="46" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C4" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="E4" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="46" t="s">
+        <v>256</v>
+      </c>
+      <c r="N4" s="46" t="s">
+        <v>275</v>
+      </c>
+      <c r="O4" s="46" t="s">
         <v>270</v>
       </c>
-      <c r="D1" s="49" t="s">
-        <v>305</v>
-      </c>
-      <c r="E1" s="49" t="s">
-        <v>306</v>
-      </c>
-      <c r="F1" s="46" t="s">
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C5" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>119</v>
+      </c>
+      <c r="E5" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="N5" s="46" t="s">
+        <v>276</v>
+      </c>
+      <c r="O5" s="46" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C6" s="46" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>119</v>
+      </c>
+      <c r="N6" s="46" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N7" s="46" t="s">
         <v>273</v>
       </c>
-      <c r="G1" s="46" t="s">
-        <v>274</v>
-      </c>
-      <c r="H1" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="I1" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="J1" s="46" t="s">
-        <v>287</v>
-      </c>
-      <c r="K1" s="46"/>
-      <c r="L1" s="50" t="s">
-        <v>117</v>
-      </c>
-      <c r="N1" s="75" t="s">
-        <v>314</v>
-      </c>
-      <c r="O1" s="48" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="C2" s="47" t="s">
-        <v>271</v>
-      </c>
-      <c r="D2" s="47" t="s">
-        <v>307</v>
-      </c>
-      <c r="E2" s="47" t="s">
-        <v>308</v>
-      </c>
-      <c r="F2" s="47" t="s">
-        <v>271</v>
-      </c>
-      <c r="G2" s="47" t="s">
-        <v>276</v>
-      </c>
-      <c r="H2" s="47" t="s">
-        <v>281</v>
-      </c>
-      <c r="I2" s="47" t="s">
-        <v>285</v>
-      </c>
-      <c r="J2" s="47" t="s">
-        <v>285</v>
-      </c>
-      <c r="L2" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" s="47" t="s">
-        <v>315</v>
-      </c>
-      <c r="O2" s="47" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="C3" s="47" t="s">
-        <v>310</v>
-      </c>
-      <c r="D3" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="E3" s="47" t="s">
-        <v>271</v>
-      </c>
-      <c r="F3" s="47" t="s">
-        <v>276</v>
-      </c>
-      <c r="G3" s="47" t="s">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N8" s="46" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N9" s="46" t="s">
         <v>277</v>
       </c>
-      <c r="H3" s="47" t="s">
-        <v>282</v>
-      </c>
-      <c r="I3" s="47" t="s">
-        <v>286</v>
-      </c>
-      <c r="J3" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="L3" s="47" t="s">
-        <v>122</v>
-      </c>
-      <c r="N3" s="47" t="s">
-        <v>301</v>
-      </c>
-      <c r="O3" s="47" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="C4" s="47" t="s">
-        <v>272</v>
-      </c>
-      <c r="D4" s="47" t="s">
-        <v>271</v>
-      </c>
-      <c r="E4" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="47" t="s">
-        <v>283</v>
-      </c>
-      <c r="N4" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="O4" s="47" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C5" s="47" t="s">
-        <v>309</v>
-      </c>
-      <c r="D5" s="47" t="s">
-        <v>134</v>
-      </c>
-      <c r="E5" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="N5" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="O5" s="47" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="C6" s="47" t="s">
-        <v>295</v>
-      </c>
-      <c r="D6" s="47" t="s">
-        <v>311</v>
-      </c>
-      <c r="E6" s="47" t="s">
-        <v>134</v>
-      </c>
-      <c r="N6" s="47" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="N7" s="47" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="N8" s="47" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="N9" s="47" t="s">
-        <v>304</v>
-      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G10" s="48" t="s">
-        <v>278</v>
+      <c r="G10" s="47" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="C11" s="47" t="s">
-        <v>275</v>
-      </c>
-      <c r="F11" s="47" t="s">
-        <v>293</v>
-      </c>
-      <c r="G11" s="47" t="s">
-        <v>291</v>
+      <c r="C11" s="46" t="s">
+        <v>248</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="G11" s="46" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="C12" s="47" t="s">
-        <v>294</v>
-      </c>
-      <c r="G12" s="47" t="s">
-        <v>289</v>
+      <c r="C12" s="46" t="s">
+        <v>267</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G13" s="47" t="s">
-        <v>290</v>
-      </c>
-      <c r="L13" s="47">
-        <v>1394.52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="L14" s="47">
-        <v>198.73</v>
-      </c>
-      <c r="M14" s="47">
-        <v>128.30000000000001</v>
+      <c r="G13" s="46" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G15" s="47" t="s">
-        <v>279</v>
-      </c>
-      <c r="L15" s="47">
-        <v>28.6</v>
-      </c>
-      <c r="M15" s="47">
-        <v>19.07</v>
+      <c r="G15" s="46" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G16" s="47" t="s">
-        <v>292</v>
-      </c>
-      <c r="L16" s="47">
-        <f>SUM(L13:L15)</f>
-        <v>1621.85</v>
-      </c>
-      <c r="M16" s="47">
-        <f>SUM(M14:M15)</f>
-        <v>147.37</v>
+      <c r="G16" s="46" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G17" s="47" t="s">
-        <v>288</v>
+      <c r="G17" s="46" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G19" s="48"/>
+      <c r="G19" s="47"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2367,430 +2238,430 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="D1" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="62"/>
-      <c r="G1" s="65" t="s">
+      <c r="A1" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="61"/>
+      <c r="D1" s="60" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="61"/>
+      <c r="G1" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="66"/>
-      <c r="J1" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="K1" s="66"/>
-      <c r="M1" s="67" t="s">
-        <v>313</v>
-      </c>
-      <c r="N1" s="68"/>
-      <c r="P1" s="63" t="s">
-        <v>250</v>
-      </c>
-      <c r="Q1" s="64"/>
+      <c r="H1" s="65"/>
+      <c r="J1" s="64" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" s="65"/>
+      <c r="M1" s="66" t="s">
+        <v>286</v>
+      </c>
+      <c r="N1" s="67"/>
+      <c r="P1" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q1" s="63"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>16</v>
-      </c>
       <c r="D2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="37" t="s">
+      <c r="G2" s="36" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="J2" s="52" t="s">
-        <v>72</v>
+        <v>61</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>71</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="M2" s="54"/>
-      <c r="N2" s="55"/>
-      <c r="P2" s="37" t="s">
-        <v>253</v>
+        <v>61</v>
+      </c>
+      <c r="M2" s="53"/>
+      <c r="N2" s="54"/>
+      <c r="P2" s="36" t="s">
+        <v>226</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="35" t="s">
         <v>9</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="M3" s="54"/>
-      <c r="N3" s="55"/>
-      <c r="P3" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="53"/>
+      <c r="N3" s="54"/>
+      <c r="P3" s="35" t="s">
         <v>9</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="M4" s="54"/>
-      <c r="N4" s="55"/>
-      <c r="P4" s="51" t="s">
-        <v>72</v>
+        <v>61</v>
+      </c>
+      <c r="M4" s="53"/>
+      <c r="N4" s="54"/>
+      <c r="P4" s="50" t="s">
+        <v>71</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="19" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" s="54"/>
-      <c r="N5" s="55"/>
+        <v>22</v>
+      </c>
+      <c r="M5" s="53"/>
+      <c r="N5" s="54"/>
       <c r="P5" s="24" t="s">
-        <v>251</v>
+        <v>224</v>
       </c>
       <c r="Q5" s="25" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>12</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>2</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" s="54"/>
-      <c r="N6" s="55"/>
+        <v>15</v>
+      </c>
+      <c r="M6" s="53"/>
+      <c r="N6" s="54"/>
       <c r="P6" s="4" t="s">
         <v>2</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>23</v>
-      </c>
       <c r="D7" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>3</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M7" s="54"/>
-      <c r="N7" s="55"/>
-      <c r="P7" s="36" t="s">
-        <v>254</v>
+        <v>15</v>
+      </c>
+      <c r="M7" s="53"/>
+      <c r="N7" s="54"/>
+      <c r="P7" s="35" t="s">
+        <v>227</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="53"/>
+      <c r="N8" s="54"/>
+      <c r="P8" s="37" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q8" s="25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="B9" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M8" s="54"/>
-      <c r="N8" s="55"/>
-      <c r="P8" s="38" t="s">
-        <v>252</v>
-      </c>
-      <c r="Q8" s="25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="45" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>39</v>
-      </c>
       <c r="E9" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G9" s="53" t="s">
-        <v>312</v>
+        <v>22</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>285</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M9" s="54"/>
-      <c r="N9" s="55"/>
+        <v>15</v>
+      </c>
+      <c r="M9" s="53"/>
+      <c r="N9" s="54"/>
       <c r="P9" s="4" t="s">
-        <v>255</v>
+        <v>228</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>7</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J10" s="29" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="K10" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="M10" s="56"/>
-      <c r="N10" s="57"/>
-      <c r="P10" s="58" t="s">
-        <v>98</v>
+        <v>94</v>
+      </c>
+      <c r="M10" s="55"/>
+      <c r="N10" s="56"/>
+      <c r="P10" s="57" t="s">
+        <v>93</v>
       </c>
       <c r="Q10" s="27" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="45" t="s">
-        <v>27</v>
+      <c r="A11" s="44" t="s">
+        <v>26</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="P11" s="58" t="s">
-        <v>312</v>
+        <v>15</v>
+      </c>
+      <c r="P11" s="57" t="s">
+        <v>285</v>
       </c>
       <c r="Q11" s="27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="32" t="s">
         <v>2</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P12" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q12" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="Q12" s="22" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
-        <v>29</v>
+      <c r="A13" s="44" t="s">
+        <v>28</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" s="30"/>
       <c r="H13" s="31"/>
       <c r="P13" s="2" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2798,344 +2669,344 @@
       <c r="B16" s="1"/>
     </row>
     <row r="17" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="61" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" s="62"/>
-      <c r="D17" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" s="62"/>
-      <c r="G17" s="59" t="s">
+      <c r="A17" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="61"/>
+      <c r="D17" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="E17" s="61"/>
+      <c r="G17" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="H17" s="60"/>
-      <c r="J17" s="59" t="s">
+      <c r="H17" s="59"/>
+      <c r="J17" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="K17" s="60"/>
-      <c r="M17" s="59" t="s">
-        <v>267</v>
-      </c>
-      <c r="N17" s="60"/>
+      <c r="K17" s="59"/>
+      <c r="M17" s="58" t="s">
+        <v>240</v>
+      </c>
+      <c r="N17" s="59"/>
       <c r="O17" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="P17" s="59" t="s">
-        <v>264</v>
-      </c>
-      <c r="Q17" s="60"/>
+        <v>237</v>
+      </c>
+      <c r="P17" s="58" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q17" s="59"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>257</v>
+        <v>58</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>230</v>
       </c>
       <c r="G18" s="12" t="s">
         <v>4</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>260</v>
+        <v>233</v>
       </c>
       <c r="N18" s="13"/>
       <c r="P18" s="4" t="s">
-        <v>265</v>
+        <v>238</v>
       </c>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="41" t="s">
-        <v>258</v>
+        <v>22</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>231</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J19" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="J19" s="43" t="s">
         <v>4</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M19" s="4" t="s">
         <v>11</v>
       </c>
       <c r="N19" s="5"/>
       <c r="P19" s="4" t="s">
-        <v>260</v>
+        <v>233</v>
       </c>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="E20" s="42" t="s">
-        <v>256</v>
+        <v>60</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>229</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>5</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J20" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K20" s="5" t="s">
-        <v>70</v>
-      </c>
       <c r="M20" s="24" t="s">
-        <v>268</v>
+        <v>241</v>
       </c>
       <c r="N20" s="25" t="s">
-        <v>269</v>
+        <v>242</v>
       </c>
       <c r="P20" s="4" t="s">
         <v>4</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>266</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>261</v>
+        <v>234</v>
       </c>
       <c r="N21" s="5"/>
       <c r="P21" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q21" s="5"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J22" s="4" t="s">
         <v>2</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>7</v>
       </c>
       <c r="N22" s="5"/>
       <c r="P22" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="Q22" s="5"/>
     </row>
     <row r="23" spans="1:17" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J23" s="4" t="s">
         <v>3</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="N23" s="43" t="s">
-        <v>262</v>
+        <v>77</v>
+      </c>
+      <c r="N23" s="42" t="s">
+        <v>235</v>
       </c>
       <c r="P23" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q23" s="7"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G24" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H24" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>7</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>263</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G25" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>259</v>
+        <v>232</v>
       </c>
       <c r="N25" s="7"/>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J26" s="24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K26" s="25" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J27" s="26" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J28" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K28" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
@@ -3177,17 +3048,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
+      <c r="B1" s="69"/>
     </row>
     <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3201,7 +3072,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>233</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3212,18 +3083,18 @@
     </row>
     <row r="6" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>234</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>235</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3231,12 +3102,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>235</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" s="34"/>
     </row>
@@ -3245,21 +3116,21 @@
         <v>7</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="34" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="B11" s="34"/>
     </row>
     <row r="12" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3267,22 +3138,22 @@
       <c r="B13" s="34"/>
     </row>
     <row r="14" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="69" t="s">
+      <c r="A14" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="70"/>
+      <c r="B14" s="69"/>
     </row>
     <row r="15" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="34"/>
     </row>
@@ -3291,35 +3162,35 @@
         <v>4</v>
       </c>
       <c r="B17" s="34" t="s">
-        <v>237</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B18" s="34"/>
     </row>
     <row r="19" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="34" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="B19" s="34"/>
     </row>
     <row r="20" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="34" t="s">
-        <v>238</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21" s="34" t="s">
-        <v>239</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3327,7 +3198,7 @@
         <v>2</v>
       </c>
       <c r="B22" s="34" t="s">
-        <v>240</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3335,7 +3206,7 @@
         <v>3</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>241</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3343,23 +3214,23 @@
         <v>7</v>
       </c>
       <c r="B24" s="34" t="s">
-        <v>242</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="34" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B25" s="34" t="s">
-        <v>188</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B26" s="34" t="s">
-        <v>243</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3367,22 +3238,22 @@
       <c r="B27" s="34"/>
     </row>
     <row r="28" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="69" t="s">
-        <v>75</v>
-      </c>
-      <c r="B28" s="70"/>
+      <c r="A28" s="68" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" s="69"/>
     </row>
     <row r="29" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30" s="34"/>
     </row>
@@ -3391,15 +3262,15 @@
         <v>11</v>
       </c>
       <c r="B31" s="34" t="s">
-        <v>244</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" s="34" t="s">
-        <v>245</v>
+        <v>219</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3407,29 +3278,29 @@
         <v>7</v>
       </c>
       <c r="B33" s="34" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B34" s="34"/>
     </row>
     <row r="35" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="34" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B35" s="34" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" s="34" t="s">
-        <v>246</v>
+        <v>220</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3437,31 +3308,31 @@
       <c r="B37" s="34"/>
     </row>
     <row r="38" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="69" t="s">
-        <v>81</v>
-      </c>
-      <c r="B38" s="70"/>
+      <c r="A38" s="68" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" s="69"/>
     </row>
     <row r="39" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B40" s="34"/>
     </row>
     <row r="41" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B41" s="34" t="s">
-        <v>247</v>
+        <v>221</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -3469,26 +3340,26 @@
         <v>4</v>
       </c>
       <c r="B42" s="34" t="s">
-        <v>248</v>
+        <v>222</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B43" s="34" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B44" s="34"/>
     </row>
     <row r="45" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B45" s="34"/>
     </row>
@@ -3506,303 +3377,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0B82FF-FA5E-4F7B-BDEC-911F80A9C9C2}">
-  <dimension ref="A1:B39"/>
-  <sheetFormatPr defaultColWidth="45.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="71.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="72"/>
-    </row>
-    <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="B2" s="33" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="34"/>
-    </row>
-    <row r="4" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="34" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="B6" s="34"/>
-    </row>
-    <row r="7" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="B11" s="34"/>
-    </row>
-    <row r="12" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-    </row>
-    <row r="16" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="71" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="72"/>
-    </row>
-    <row r="17" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="B17" s="33" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="34"/>
-    </row>
-    <row r="19" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="34" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="34" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="34"/>
-    </row>
-    <row r="24" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="34" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="B25" s="34" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="B26" s="34"/>
-    </row>
-    <row r="27" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="34"/>
-      <c r="B27" s="34"/>
-    </row>
-    <row r="28" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="71" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="72"/>
-    </row>
-    <row r="29" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="B29" s="33" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="B30" s="34"/>
-    </row>
-    <row r="31" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" s="34" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" s="34" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="B33" s="34" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="B34" s="34"/>
-    </row>
-    <row r="35" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="B35" s="34" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="B36" s="34" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="B37" s="34" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="34" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="34"/>
-      <c r="B39" s="34"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A28:B28"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{169BDFE5-2040-421E-ADD6-99433B28DF6E}">
   <dimension ref="A1:B99"/>
   <sheetFormatPr defaultColWidth="38.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3812,40 +3386,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="s">
-        <v>189</v>
-      </c>
-      <c r="B1" s="74"/>
+      <c r="A1" s="70" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="71"/>
     </row>
     <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B3" s="34"/>
     </row>
     <row r="4" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="34" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="B4" s="34"/>
     </row>
     <row r="5" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
-        <v>191</v>
+        <v>169</v>
       </c>
       <c r="B5" s="34"/>
     </row>
     <row r="6" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B6" s="34"/>
     </row>
@@ -3854,17 +3428,17 @@
       <c r="B7" s="34"/>
     </row>
     <row r="8" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="73" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="74"/>
+      <c r="A8" s="70" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="71"/>
     </row>
     <row r="9" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3875,112 +3449,112 @@
     </row>
     <row r="11" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="34" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="B11" s="34" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="34" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="34" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="B13" s="34" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="34" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="34" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="34" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B16" s="34" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="34" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="B17" s="34" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="34" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B19" s="34" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="34" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="B20" s="34" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="34" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="B21" s="34" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
-        <v>194</v>
+        <v>172</v>
       </c>
       <c r="B22" s="34"/>
     </row>
     <row r="23" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="34" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="34" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="B24" s="34" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3988,70 +3562,70 @@
       <c r="B25" s="34"/>
     </row>
     <row r="26" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="73" t="s">
-        <v>195</v>
-      </c>
-      <c r="B26" s="74"/>
+      <c r="A26" s="70" t="s">
+        <v>173</v>
+      </c>
+      <c r="B26" s="71"/>
     </row>
     <row r="27" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="34" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="B28" s="34"/>
     </row>
     <row r="29" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="34" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="B29" s="34"/>
     </row>
     <row r="30" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="B30" s="34"/>
     </row>
     <row r="31" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="34" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="B31" s="34"/>
     </row>
     <row r="32" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="34" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="B32" s="34"/>
     </row>
     <row r="33" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="34" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="B33" s="34"/>
     </row>
     <row r="34" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="34" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="B34" s="34"/>
     </row>
     <row r="35" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="34" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="B35" s="34"/>
     </row>
     <row r="36" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="34" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B36" s="34"/>
     </row>
@@ -4060,147 +3634,147 @@
       <c r="B37" s="34"/>
     </row>
     <row r="38" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="73" t="s">
-        <v>143</v>
-      </c>
-      <c r="B38" s="74"/>
+      <c r="A38" s="70" t="s">
+        <v>128</v>
+      </c>
+      <c r="B38" s="71"/>
     </row>
     <row r="39" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="34"/>
     </row>
     <row r="41" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="34" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="B41" s="34" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="34" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B42" s="34" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="34" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B43" s="34" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B44" s="34"/>
     </row>
     <row r="45" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="34" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="B45" s="34" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="34" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B46" s="34" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="34" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="B47" s="34" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="34" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="B48" s="34"/>
     </row>
     <row r="49" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="34" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="B49" s="34" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="34" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="B50" s="34" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="34" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="B51" s="34" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="34" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="B52" s="34" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="34" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="B53" s="34" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="34" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="B54" s="34" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="34" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="B55" s="34" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B56" s="34" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4208,46 +3782,46 @@
       <c r="B57" s="34"/>
     </row>
     <row r="58" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="73" t="s">
-        <v>207</v>
-      </c>
-      <c r="B58" s="74"/>
+      <c r="A58" s="70" t="s">
+        <v>185</v>
+      </c>
+      <c r="B58" s="71"/>
     </row>
     <row r="59" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B59" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="34" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="B60" s="34"/>
     </row>
     <row r="61" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="34" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="B61" s="34"/>
     </row>
     <row r="62" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="34" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="B62" s="34"/>
     </row>
     <row r="63" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="34" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="B63" s="34"/>
     </row>
     <row r="64" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B64" s="34"/>
     </row>
@@ -4256,50 +3830,50 @@
       <c r="B65" s="34"/>
     </row>
     <row r="66" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="73" t="s">
-        <v>169</v>
-      </c>
-      <c r="B66" s="74"/>
+      <c r="A66" s="70" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="71"/>
     </row>
     <row r="67" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B67" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="34" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B68" s="34"/>
     </row>
     <row r="69" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="34" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="B69" s="34" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B70" s="34"/>
     </row>
     <row r="71" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="34" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="B71" s="34" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B72" s="34"/>
     </row>
@@ -4308,64 +3882,64 @@
       <c r="B73" s="34"/>
     </row>
     <row r="74" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="B74" s="74"/>
+      <c r="A74" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="B74" s="71"/>
     </row>
     <row r="75" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B75" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="34" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="B76" s="34"/>
     </row>
     <row r="77" spans="1:2" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="34" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B77" s="34" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B78" s="34" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="158.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="34" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="B79" s="34" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="34" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="B80" s="34"/>
     </row>
     <row r="81" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="34" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="B81" s="34"/>
     </row>
     <row r="82" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B82" s="34"/>
     </row>
@@ -4374,22 +3948,22 @@
       <c r="B83" s="34"/>
     </row>
     <row r="84" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="73" t="s">
-        <v>171</v>
-      </c>
-      <c r="B84" s="74"/>
+      <c r="A84" s="70" t="s">
+        <v>156</v>
+      </c>
+      <c r="B84" s="71"/>
     </row>
     <row r="85" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B85" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="34" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="B86" s="34"/>
     </row>
@@ -4398,38 +3972,38 @@
         <v>11</v>
       </c>
       <c r="B87" s="34" t="s">
-        <v>221</v>
+        <v>199</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="34" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B88" s="34" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="34" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="B89" s="34"/>
     </row>
     <row r="90" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="34" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="B90" s="34"/>
     </row>
     <row r="91" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="34" t="s">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="B91" s="34"/>
     </row>
     <row r="92" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="34" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B92" s="34"/>
     </row>
@@ -4438,39 +4012,39 @@
       <c r="B93" s="34"/>
     </row>
     <row r="94" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="73" t="s">
-        <v>175</v>
-      </c>
-      <c r="B94" s="74"/>
+      <c r="A94" s="70" t="s">
+        <v>160</v>
+      </c>
+      <c r="B94" s="71"/>
     </row>
     <row r="95" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="33" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B95" s="33" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="34" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="B96" s="34"/>
     </row>
     <row r="97" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="34" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="B97" s="34" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B98" s="34" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4478,7 +4052,7 @@
         <v>2</v>
       </c>
       <c r="B99" s="34" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added custom columns and used it for items and orderlines
</commit_message>
<xml_diff>
--- a/docs/BPS Tables.xlsx
+++ b/docs/BPS Tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\orderNexa\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE16BB2C-B581-4346-A222-67C1321C9504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6905321C-FEB6-46CC-8E5D-6AC513482176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{04488C40-F022-43DD-81A9-CABA93E3C950}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="309">
   <si>
     <t>ar_transactions</t>
   </si>
@@ -928,6 +928,45 @@
   </si>
   <si>
     <t>price</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>value_type</t>
+  </si>
+  <si>
+    <t>sort_order</t>
+  </si>
+  <si>
+    <t>fnd_tenant_options</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (1, 1001, 'SLICED',          'Sliced',          'boolean', 10, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1002, 'WRAPPED',         'Wrapped',         'boolean', 20, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1003, 'COVERED',         'Covered',         'boolean', 30, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1004, 'SPRINKLES_COLOR', 'Sprinkles Color', 'text',    40, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1005, 'MESSAGE_TEXT',    'Message Text',    'text',    50, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1006, 'CANDLE_COUNT',    'Candle Count',    'number',  60, true),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (1, 1007, 'RUSH_PREP',       'Rush Prep',       'boolean', 70, false);</t>
+  </si>
+  <si>
+    <t>tenant_option_id</t>
+  </si>
+  <si>
+    <t>option_code</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1551,13 +1590,18 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2252,66 +2296,134 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31DB8649-7856-4099-8378-0669DC3CA052}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21" style="74" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="74"/>
-    <col min="5" max="5" width="31.85546875" style="74" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="74"/>
-    <col min="7" max="7" width="16.85546875" style="74" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="74"/>
+    <col min="1" max="1" width="21" style="75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="75"/>
+    <col min="3" max="3" width="31.85546875" style="75" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.140625" style="73" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.140625" style="73"/>
+    <col min="9" max="9" width="52.140625" style="73" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="73"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="74" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="74" t="s">
         <v>290</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="C1" s="76" t="s">
         <v>154</v>
       </c>
-      <c r="F1" s="76"/>
-      <c r="G1" s="73" t="s">
+      <c r="D1" s="74" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="74" t="s">
+      <c r="E1" s="77" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="75" t="s">
         <v>293</v>
       </c>
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="74" t="s">
+      <c r="C2" s="75" t="s">
         <v>291</v>
       </c>
-      <c r="G2" s="74" t="s">
+      <c r="D2" s="75" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="74" t="s">
+      <c r="E2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="75" t="s">
         <v>291</v>
       </c>
-      <c r="E3" s="74" t="s">
+      <c r="C3" s="75" t="s">
         <v>294</v>
       </c>
-      <c r="G3" s="74" t="s">
+      <c r="D3" s="75" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G4" s="74" t="s">
+      <c r="E3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="D4" s="75" t="s">
         <v>295</v>
       </c>
+      <c r="E4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E9"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E12" s="73" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E13" s="73" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E14" s="73" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E15" s="73" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E16" s="73" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="73" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="73" t="s">
+        <v>306</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="E1:F1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>